<commit_message>
balance-xlsx: workbook-driven category exclusions on dashboard + insights
The Constants sheet gains an optional "Excluded from Budget by Default" list; the Budgets block and the new list share a canonical position to the right of the category table, and both are read from anywhere and migrated there on the next settings save (fixing legacy placements like the current row ~1000 one).

Server: /data accepts repeated exclude params (view override of the workbook defaults) and returns defaultExcludedCategories; POST /excluded-defaults writes the list back; budget notifications inherit the defaults. UI: the dashboard gets a categories dialog reusing the insights checkbox panels with reset + save-as-default; insights seeds its per-currency exclusions from conversions plus the workbook defaults.
</commit_message>
<xml_diff>
--- a/apps/balance-xlsx/mock-data.xlsx
+++ b/apps/balance-xlsx/mock-data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="75">
   <si>
     <t>Date</t>
   </si>
@@ -158,6 +158,9 @@
     <t>Symbols</t>
   </si>
   <si>
+    <t>Budgets</t>
+  </si>
+  <si>
     <t>School Fees</t>
   </si>
   <si>
@@ -167,6 +170,12 @@
     <t>$</t>
   </si>
   <si>
+    <t>Monthly Budget</t>
+  </si>
+  <si>
+    <t>First Day Bias</t>
+  </si>
+  <si>
     <t>Clothes</t>
   </si>
   <si>
@@ -203,6 +212,9 @@
     <t>Loan</t>
   </si>
   <si>
+    <t>Excluded from Budget by Default</t>
+  </si>
+  <si>
     <t>Food General</t>
   </si>
   <si>
@@ -225,15 +237,6 @@
   </si>
   <si>
     <t>Medical</t>
-  </si>
-  <si>
-    <t>Budgets</t>
-  </si>
-  <si>
-    <t>Monthly Budget</t>
-  </si>
-  <si>
-    <t>First Day Bias</t>
   </si>
 </sst>
 </file>
@@ -3244,7 +3247,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -3255,7 +3258,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>42</v>
       </c>
@@ -3277,51 +3280,72 @@
       <c r="G2" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="I2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="C3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
         <v>24</v>
       </c>
       <c r="G4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="I4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="3">
+        <v>3000</v>
+      </c>
+      <c r="K4" s="3">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -3329,10 +3353,10 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
         <v>31</v>
@@ -3340,49 +3364,67 @@
       <c r="G5" t="s">
         <v>10</v>
       </c>
+      <c r="I5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" s="3">
+        <v>500</v>
+      </c>
+      <c r="K5" s="3">
+        <v>100</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+      <c r="I7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D8" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D9" t="s">
-        <v>66</v>
+        <v>70</v>
+      </c>
+      <c r="I9" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3390,58 +3432,20 @@
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="3">
-        <v>3000</v>
-      </c>
-      <c r="C17" s="3">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="3">
-        <v>500</v>
-      </c>
-      <c r="C18" s="3">
-        <v>100</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
balance-xlsx: settings blocks adopt the table's cell styles
The Budgets and Excluded blocks now copy the header/body styles from the first category-table columns when written, so their fonts, borders and fills match the surrounding sheet instead of falling back to the workbook default (or leftover styles). The mock generator styles the budget header per cell instead of the whole row.
</commit_message>
<xml_diff>
--- a/apps/balance-xlsx/mock-data.xlsx
+++ b/apps/balance-xlsx/mock-data.xlsx
@@ -3284,26 +3284,26 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
         <v>51</v>
       </c>
       <c r="I3" s="1" t="s">

</xml_diff>